<commit_message>
Publish fully audited college production cluster
</commit_message>
<xml_diff>
--- a/college-production-tracker.xlsx
+++ b/college-production-tracker.xlsx
@@ -1409,27 +1409,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
     </row>

</xml_diff>